<commit_message>
feat: actions column ("<qty> to <step>"); drop rows covered by finished stock
- Result sheet's "next step" column is now "actions", e.g. "58 to Edge and drill".
- Finished (300) stock only counts when it covers the qty asked for in the
  email; such rows are dropped from the reply. Short rows route on 310/400.
- New pure helpers formatAction() / buildResultRows() above the glue marker,
  with tests (14/14). independent_check.py updated with the same rule.
- input-mixed.xlsx gains two finished-stock edge rows (short, exactly equal);
  both expected-output files regenerated. README updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XAdenmSZVcpJJ8ChNNUTtK
</commit_message>
<xml_diff>
--- a/sample/expected-output-mixed.xlsx
+++ b/sample/expected-output-mixed.xlsx
@@ -434,107 +434,107 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>next step</t>
+          <t>actions</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>30010482731</t>
+          <t>30040995108</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>18 Wte 600x900 CAD-104827</t>
+          <t>18 Anth 651x824 CAD-409951</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>25</v>
+        <v>117</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Finished, no action</t>
+          <t>117 to Drill</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>30040995108</t>
+          <t>30026196225</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>18 Anth 651x824 CAD-409951</t>
+          <t>18 Oak 662x854 CAD-261962</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>117</v>
+        <v>58</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Drill</t>
+          <t>58 to Edge and drill</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>30026196225</t>
+          <t>30061891516</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>18 Oak 662x854 CAD-261962</t>
+          <t>18 Wte 415x947 CAD-618915</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Edge and drill</t>
+          <t>59 to Cut, edge and drill</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>30061891516</t>
+          <t>30099999999</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>18 Wte 415x947 CAD-618915</t>
+          <t>Tiled Panel (unknown SKU test row)</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>59</v>
+        <v>1</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Cut, edge and drill</t>
+          <t>1 to SKU NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>30099999999</t>
+          <t>30094410887</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tiled Panel (unknown SKU test row)</t>
+          <t>18 Oak 408x960 CAD-944108</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>SKU NOT FOUND</t>
+          <t>100 to Edge and drill</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: drop qty column from result sheet; qty lives in actions
Result columns are now sku, description, actions. independent_check.py
also checks the header; expected-output samples regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XAdenmSZVcpJJ8ChNNUTtK
</commit_message>
<xml_diff>
--- a/sample/expected-output-mixed.xlsx
+++ b/sample/expected-output-mixed.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,11 +429,6 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>qty</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
           <t>actions</t>
         </is>
       </c>
@@ -449,10 +444,7 @@
           <t>18 Anth 651x824 CAD-409951</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>117</v>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>117 to Drill</t>
         </is>
@@ -469,10 +461,7 @@
           <t>18 Oak 662x854 CAD-261962</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>58</v>
-      </c>
-      <c r="D3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>58 to Edge and drill</t>
         </is>
@@ -489,10 +478,7 @@
           <t>18 Wte 415x947 CAD-618915</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>59</v>
-      </c>
-      <c r="D4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>59 to Cut, edge and drill</t>
         </is>
@@ -509,10 +495,7 @@
           <t>Tiled Panel (unknown SKU test row)</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>SKU NOT FOUND</t>
         </is>
@@ -529,10 +512,7 @@
           <t>18 Oak 408x960 CAD-944108</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>100</v>
-      </c>
-      <c r="D6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>100 to Edge and drill</t>
         </is>

</xml_diff>

<commit_message>
feat: result xlsx has borders on every cell and columns sized to fit
Build xlsx is now a Code node (buildXlsx writes the xlsx parts and zips
them, stored) since Convert to File can't set widths or borders and the
Code node can't load an xlsx library without changing n8n settings.
tests/xlsx.test.js covers it; independent_check.py checks the layout and
--write formats the samples the same way.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XAdenmSZVcpJJ8ChNNUTtK
</commit_message>
<xml_diff>
--- a/sample/expected-output-mixed.xlsx
+++ b/sample/expected-output-mixed.xlsx
@@ -34,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +42,19 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -415,104 +422,109 @@
   </sheetPr>
   <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>sku</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>actions</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>30040995108</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>18 Anth 651x824 CAD-409951</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>117 to Drill</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>30026196225</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>18 Oak 662x854 CAD-261962</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>58 to Edge and drill</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>30061891516</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>18 Wte 415x947 CAD-618915</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>59 to Cut, edge and drill</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>30099999999</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>Tiled Panel (unknown SKU test row)</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>SKU NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>30094410887</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>18 Oak 408x960 CAD-944108</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>100 to Edge and drill</t>
         </is>

</xml_diff>